<commit_message>
Fact-check fixes: Nebius correction passage, sources and multiple
Logged in research-build/CHANGELOG.md. No call, scenario value or revisit
level changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/research/2026-10-06_Nebius_Model.xlsx
+++ b/public/research/2026-10-06_Nebius_Model.xlsx
@@ -937,19 +937,19 @@
     <t xml:space="preserve">2027 EBITDA, US$bn, unrounded</t>
   </si>
   <si>
-    <t xml:space="preserve">2027 EBITDA, US$bn, as stated in the pitch (rounded)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV / 2027 EBITDA, as in the pitch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pitch: about 12.6x on ~US$6.2bn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV / 2027 EBITDA, on unrounded EBITDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same thing before rounding; shown for transparency</t>
+    <t xml:space="preserve">2027 EBITDA, US$bn, rounded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / 2027 EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: about 12.7x on ~US$6.15bn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / 2027 EBITDA, on rounded EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shown for transparency</t>
   </si>
   <si>
     <t xml:space="preserve">EV / 2027 revenue</t>
@@ -4409,8 +4409,8 @@
         <v>303</v>
       </c>
       <c r="B10" s="42" t="n">
-        <f aca="false">B5/B9</f>
-        <v>12.5791740471848</v>
+        <f aca="false">B5/B8</f>
+        <v>12.6814437548855</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>304</v>
@@ -4421,8 +4421,8 @@
         <v>305</v>
       </c>
       <c r="B11" s="22" t="n">
-        <f aca="false">B5/B8</f>
-        <v>12.6814437548855</v>
+        <f aca="false">B5/B9</f>
+        <v>12.5791740471848</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>306</v>

</xml_diff>